<commit_message>
Verified Chinese names + bulletproof drawer (fixed-height transform-only)
</commit_message>
<xml_diff>
--- a/data/HK_Vegetarian_Restaurants_Database.xlsx
+++ b/data/HK_Vegetarian_Restaurants_Database.xlsx
@@ -1376,7 +1376,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8½ Otto e Mezzo Bombana</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -4616,7 +4616,7 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>சரவணபவன்</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -5336,7 +5336,7 @@
       </c>
       <c r="D41" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>李好純</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
@@ -7256,7 +7256,7 @@
       </c>
       <c r="D57" s="13" t="inlineStr">
         <is>
-          <t>龍門樓 / 志蓮素齋</t>
+          <t>志蓮素齋</t>
         </is>
       </c>
       <c r="E57" s="13" t="inlineStr">
@@ -7976,7 +7976,7 @@
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>遊</t>
+          <t>游°</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
@@ -8456,7 +8456,7 @@
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>爵樂印度餐廳</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
@@ -12296,7 +12296,7 @@
       </c>
       <c r="D99" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>光線素食</t>
         </is>
       </c>
       <c r="E99" s="13" t="inlineStr">
@@ -13909,7 +13909,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8½ Otto e Mezzo Bombana</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -17149,7 +17149,7 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>சரவணபவன்</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -17869,7 +17869,7 @@
       </c>
       <c r="D41" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>李好純</t>
         </is>
       </c>
       <c r="E41" s="13" t="inlineStr">
@@ -19789,7 +19789,7 @@
       </c>
       <c r="D57" s="13" t="inlineStr">
         <is>
-          <t>龍門樓 / 志蓮素齋</t>
+          <t>志蓮素齋</t>
         </is>
       </c>
       <c r="E57" s="13" t="inlineStr">
@@ -20509,7 +20509,7 @@
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>遊</t>
+          <t>游°</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
@@ -20989,7 +20989,7 @@
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>爵樂印度餐廳</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
@@ -24829,7 +24829,7 @@
       </c>
       <c r="D99" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>光線素食</t>
         </is>
       </c>
       <c r="E99" s="13" t="inlineStr">
@@ -25962,7 +25962,7 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>李好純</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
@@ -26442,7 +26442,7 @@
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>龍門樓 / 志蓮素齋</t>
+          <t>志蓮素齋</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
@@ -26682,7 +26682,7 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>遊</t>
+          <t>游°</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
@@ -28962,7 +28962,7 @@
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>光線素食</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">
@@ -32908,7 +32908,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8½ Otto e Mezzo Bombana</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -36801,7 +36801,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>சரவணபவன்</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -37521,7 +37521,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>爵樂印度餐廳</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">

</xml_diff>